<commit_message>
I gave up on commiting this cleanly
</commit_message>
<xml_diff>
--- a/utils/tstart-tend.xlsx
+++ b/utils/tstart-tend.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26731"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27928"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\leroquan\Documents\python\preprocessing-mitgcm\utils\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47616D3D-7FDE-425C-8B08-A8594F24E89C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80384A03-15F5-4BA0-AA04-6F8B4F74E925}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11620" activeTab="4" xr2:uid="{1C1AAA8F-B7A7-4F2E-9366-9D04187454FC}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="7" xr2:uid="{1C1AAA8F-B7A7-4F2E-9366-9D04187454FC}"/>
   </bookViews>
   <sheets>
     <sheet name="13.08.2023" sheetId="1" r:id="rId1"/>
@@ -19,6 +19,8 @@
     <sheet name="01.03.2024" sheetId="3" r:id="rId4"/>
     <sheet name="01.03.2025" sheetId="7" r:id="rId5"/>
     <sheet name="01.12.2023" sheetId="2" r:id="rId6"/>
+    <sheet name="01.01.2026" sheetId="8" r:id="rId7"/>
+    <sheet name="01.01.2025" sheetId="9" r:id="rId8"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -41,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="9">
   <si>
     <t xml:space="preserve">Tstart = </t>
   </si>
@@ -126,9 +128,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -166,7 +168,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -272,7 +274,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -414,7 +416,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1250,4 +1252,270 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{64AFCAA9-526B-4BBB-A223-4908A7BA875E}">
+  <dimension ref="B2:G12"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="2" max="2" width="14.26953125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.54296875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.54296875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C2" s="3">
+        <f>G2</f>
+        <v>46023</v>
+      </c>
+      <c r="F2" t="s">
+        <v>2</v>
+      </c>
+      <c r="G2" s="3">
+        <v>46023</v>
+      </c>
+    </row>
+    <row r="3" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C3" s="1">
+        <f>G3</f>
+        <v>10</v>
+      </c>
+      <c r="F3" t="s">
+        <v>3</v>
+      </c>
+      <c r="G3" s="1">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B4" t="s">
+        <v>0</v>
+      </c>
+      <c r="C4" s="1">
+        <v>4752000</v>
+      </c>
+      <c r="F4" t="s">
+        <v>7</v>
+      </c>
+      <c r="G4" s="3">
+        <v>45770</v>
+      </c>
+    </row>
+    <row r="5" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B5" t="s">
+        <v>1</v>
+      </c>
+      <c r="C5">
+        <v>23760000</v>
+      </c>
+      <c r="F5" t="s">
+        <v>8</v>
+      </c>
+      <c r="G5" s="3">
+        <v>45962</v>
+      </c>
+    </row>
+    <row r="6" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B6" t="s">
+        <v>4</v>
+      </c>
+      <c r="C6">
+        <v>198540</v>
+      </c>
+    </row>
+    <row r="8" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="F8" t="s">
+        <v>0</v>
+      </c>
+      <c r="G8" s="1">
+        <f>(G4-$G$2)*24*60*60</f>
+        <v>-21859200</v>
+      </c>
+    </row>
+    <row r="9" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B9" t="s">
+        <v>7</v>
+      </c>
+      <c r="C9" s="2">
+        <f>$C$2+C4/(24*60*60)</f>
+        <v>46078</v>
+      </c>
+      <c r="F9" t="s">
+        <v>5</v>
+      </c>
+      <c r="G9" s="1">
+        <f>(G5-$G$2)*24*60*60</f>
+        <v>-5270400</v>
+      </c>
+    </row>
+    <row r="10" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B10" t="s">
+        <v>8</v>
+      </c>
+      <c r="C10" s="2">
+        <f>$C$2+C5/(24*60*60)</f>
+        <v>46298</v>
+      </c>
+    </row>
+    <row r="11" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="F11" t="s">
+        <v>4</v>
+      </c>
+      <c r="G11">
+        <f>G8/$G$3</f>
+        <v>-2185920</v>
+      </c>
+    </row>
+    <row r="12" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B12" t="s">
+        <v>6</v>
+      </c>
+      <c r="C12" s="3">
+        <f>$C$2+C6/(24*60*60)*C3</f>
+        <v>46045.979166666664</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4B99AB26-8EB3-493A-9F6D-78FC21FACCDC}">
+  <dimension ref="B2:G12"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="2" max="2" width="14.26953125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.54296875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.54296875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C2" s="3">
+        <f>G2</f>
+        <v>45658</v>
+      </c>
+      <c r="F2" t="s">
+        <v>2</v>
+      </c>
+      <c r="G2" s="3">
+        <v>45658</v>
+      </c>
+    </row>
+    <row r="3" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C3" s="1">
+        <f>G3</f>
+        <v>7</v>
+      </c>
+      <c r="F3" t="s">
+        <v>3</v>
+      </c>
+      <c r="G3" s="1">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="4" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B4" t="s">
+        <v>0</v>
+      </c>
+      <c r="C4" s="1">
+        <v>4752000</v>
+      </c>
+      <c r="F4" t="s">
+        <v>7</v>
+      </c>
+      <c r="G4" s="3">
+        <v>45770</v>
+      </c>
+    </row>
+    <row r="5" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B5" t="s">
+        <v>1</v>
+      </c>
+      <c r="C5">
+        <v>23760000</v>
+      </c>
+      <c r="F5" t="s">
+        <v>8</v>
+      </c>
+      <c r="G5" s="3">
+        <v>45962</v>
+      </c>
+    </row>
+    <row r="6" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B6" t="s">
+        <v>4</v>
+      </c>
+      <c r="C6">
+        <v>4492800</v>
+      </c>
+    </row>
+    <row r="8" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="F8" t="s">
+        <v>0</v>
+      </c>
+      <c r="G8" s="1">
+        <f>(G4-$G$2)*24*60*60</f>
+        <v>9676800</v>
+      </c>
+    </row>
+    <row r="9" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B9" t="s">
+        <v>7</v>
+      </c>
+      <c r="C9" s="2">
+        <f>$C$2+C4/(24*60*60)</f>
+        <v>45713</v>
+      </c>
+      <c r="F9" t="s">
+        <v>5</v>
+      </c>
+      <c r="G9" s="1">
+        <f>(G5-$G$2)*24*60*60</f>
+        <v>26265600</v>
+      </c>
+    </row>
+    <row r="10" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B10" t="s">
+        <v>8</v>
+      </c>
+      <c r="C10" s="2">
+        <f>$C$2+C5/(24*60*60)</f>
+        <v>45933</v>
+      </c>
+    </row>
+    <row r="11" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="F11" t="s">
+        <v>4</v>
+      </c>
+      <c r="G11">
+        <f>G8/$G$3</f>
+        <v>1382400</v>
+      </c>
+    </row>
+    <row r="12" spans="2:7" x14ac:dyDescent="0.35">
+      <c r="B12" t="s">
+        <v>6</v>
+      </c>
+      <c r="C12" s="3">
+        <f>$C$2+C6/(24*60*60)*C3</f>
+        <v>46022</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>